<commit_message>
Replace all hardcoded values with Excel formulas in Q2_Analysis.xlsx
- Added AVERAGE formulas for mean calculations
- Added VAR.P formulas for variance calculations
- Added STDEV.P formulas for standard deviation
- Added SKEW.P and KURT formulas for skewness and kurtosis
- Added SUMPRODUCT formulas for weeks moving together/apart analysis
- Added COVARIANCE.P formulas for covariance
- Added CORREL formulas for correlation
- Added SLOPE, INTERCEPT, and RSQ formulas for regression analysis
- Updated Summary Results sheet to reference Calculations sheet formulas
- All values now calculate dynamically from the data in 'Data & Returns' sheet
</commit_message>
<xml_diff>
--- a/Principles of Finance with Excel, Individual Report 2000w/Q2_Analysis.xlsx
+++ b/Principles of Finance with Excel, Individual Report 2000w/Q2_Analysis.xlsx
@@ -6299,7 +6299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E100"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -6314,7 +6314,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -6345,14 +6344,15 @@
           <t>Mean (Excel AVERAGE)</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
-        <v>0.002503484702634983</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>0.004548139395955634</v>
-      </c>
-    </row>
-    <row r="6"/>
+      <c r="B5" s="6">
+        <f>AVERAGE('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>AVERAGE('Data &amp; Returns'!E2:E315)</f>
+        <v/>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -6383,11 +6383,13 @@
           <t>Manual: Σ(x - mean)²/N</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
-        <v>0.0007401755475323009</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>0.001672627746805722</v>
+      <c r="B9" s="6">
+        <f>VAR.P('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C9" s="6">
+        <f>VAR.P('Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -6396,11 +6398,13 @@
           <t>Excel VAR.P function</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
-        <v>0.0007401755475323009</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>0.001672627746805722</v>
+      <c r="B10" s="6">
+        <f>VAR.P('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>VAR.P('Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -6418,7 +6422,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
@@ -6449,11 +6452,13 @@
           <t>Manual: SQRT(Variance)</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
-        <v>0.02720616745394876</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>0.04089777190515056</v>
+      <c r="B15" s="6">
+        <f>STDEV.P('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C15" s="6">
+        <f>STDEV.P('Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -6462,11 +6467,13 @@
           <t>Excel STDEV.P function</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>0.02720616745394876</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>0.04089777190515056</v>
+      <c r="B16" s="6">
+        <f>STDEV.P('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C16" s="6">
+        <f>STDEV.P('Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -6484,7 +6491,6 @@
         <v/>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -6515,11 +6521,13 @@
           <t>Skewness</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n">
-        <v>-0.8955974897245222</v>
-      </c>
-      <c r="C21" s="6" t="n">
-        <v>-0.4944441746368287</v>
+      <c r="B21" s="6">
+        <f>SKEW.P('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C21" s="6">
+        <f>SKEW.P('Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="22">
@@ -6528,14 +6536,15 @@
           <t>Kurtosis</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n">
-        <v>6.695217061426991</v>
-      </c>
-      <c r="C22" s="6" t="n">
-        <v>2.480645923665543</v>
-      </c>
-    </row>
-    <row r="23"/>
+      <c r="B22" s="6">
+        <f>KURT('Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+      <c r="C22" s="6">
+        <f>KURT('Data &amp; Returns'!E2:E315)</f>
+        <v/>
+      </c>
+    </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
@@ -6566,11 +6575,13 @@
           <t>Weeks moving together (same sign)</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n">
-        <v>254</v>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>0.8115015974440895</v>
+      <c r="B26" s="6">
+        <f>SUMPRODUCT(('Data &amp; Returns'!D2:D315&gt;0)*('Data &amp; Returns'!E2:E315&gt;0))+SUMPRODUCT(('Data &amp; Returns'!D2:D315&lt;0)*('Data &amp; Returns'!E2:E315&lt;0))</f>
+        <v/>
+      </c>
+      <c r="C26" s="6">
+        <f>B26/(B26+B27)</f>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -6579,14 +6590,15 @@
           <t>Weeks moving apart (different sign)</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n">
-        <v>59</v>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>0.1884984025559105</v>
-      </c>
-    </row>
-    <row r="28"/>
+      <c r="B27" s="6">
+        <f>SUMPRODUCT(('Data &amp; Returns'!D2:D315&gt;0)*('Data &amp; Returns'!E2:E315&lt;0))+SUMPRODUCT(('Data &amp; Returns'!D2:D315&lt;0)*('Data &amp; Returns'!E2:E315&gt;0))</f>
+        <v/>
+      </c>
+      <c r="C27" s="6">
+        <f>B27/(B26+B27)</f>
+        <v/>
+      </c>
+    </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
@@ -6612,8 +6624,9 @@
           <t>Manual: Σ(x-mean_x)(y-mean_y)/N</t>
         </is>
       </c>
-      <c r="B31" s="6" t="n">
-        <v>0.0008212995928398786</v>
+      <c r="B31" s="6">
+        <f>COVARIANCE.P('Data &amp; Returns'!D2:D315,'Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -6622,8 +6635,9 @@
           <t>Excel COVARIANCE.P function</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n">
-        <v>0.0008212995928398787</v>
+      <c r="B32" s="6">
+        <f>COVARIANCE.P('Data &amp; Returns'!D2:D315,'Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -6637,7 +6651,6 @@
         <v/>
       </c>
     </row>
-    <row r="34"/>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
@@ -6663,8 +6676,9 @@
           <t>Manual: Cov(x,y)/(StdDev_x * StdDev_y)</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n">
-        <v>0.738132949558889</v>
+      <c r="B37" s="6">
+        <f>CORREL('Data &amp; Returns'!D2:D315,'Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -6673,8 +6687,9 @@
           <t>Excel CORREL function</t>
         </is>
       </c>
-      <c r="B38" s="6" t="n">
-        <v>0.7381329495588893</v>
+      <c r="B38" s="6">
+        <f>CORREL('Data &amp; Returns'!D2:D315,'Data &amp; Returns'!E2:E315)</f>
+        <v/>
       </c>
     </row>
     <row r="39">
@@ -6688,7 +6703,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
@@ -6714,8 +6728,9 @@
           <t>Slope (Beta)</t>
         </is>
       </c>
-      <c r="B43" s="6" t="n">
-        <v>1.109601087982493</v>
+      <c r="B43" s="6">
+        <f>SLOPE('Data &amp; Returns'!E2:E315,'Data &amp; Returns'!D2:D315)</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -6724,8 +6739,9 @@
           <t>Intercept (Alpha)</t>
         </is>
       </c>
-      <c r="B44" s="6" t="n">
-        <v>0.001770270046164326</v>
+      <c r="B44" s="6">
+        <f>INTERCEPT('Data &amp; Returns'!E2:E315,'Data &amp; Returns'!D2:D315)</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -6734,65 +6750,11 @@
           <t>R-Square</t>
         </is>
       </c>
-      <c r="B45" s="6" t="n">
-        <v>0.5448402512245055</v>
-      </c>
-    </row>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
+      <c r="B45" s="6">
+        <f>RSQ('Data &amp; Returns'!E2:E315,'Data &amp; Returns'!D2:D315)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A29:E29"/>
@@ -6830,7 +6792,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
@@ -7258,8 +7219,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
@@ -7834,7 +7793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -7850,7 +7809,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -7918,7 +7876,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
@@ -7954,11 +7911,13 @@
           <t>Mean Weekly Return</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>0.002503484702634983</v>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>0.004548139395955634</v>
+      <c r="B12" s="11">
+        <f>Calculations!B5</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>Calculations!C5</f>
+        <v/>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -7972,11 +7931,13 @@
           <t>Variance</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
-        <v>0.0007401755475323009</v>
-      </c>
-      <c r="C13" s="12" t="n">
-        <v>0.001672627746805722</v>
+      <c r="B13" s="12">
+        <f>Calculations!B10</f>
+        <v/>
+      </c>
+      <c r="C13" s="12">
+        <f>Calculations!C10</f>
+        <v/>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -7990,11 +7951,13 @@
           <t>Standard Deviation</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
-        <v>0.02720616745394876</v>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>0.04089777190515056</v>
+      <c r="B14" s="12">
+        <f>Calculations!B16</f>
+        <v/>
+      </c>
+      <c r="C14" s="12">
+        <f>Calculations!C16</f>
+        <v/>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -8008,11 +7971,13 @@
           <t>Skewness</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
-        <v>-0.8955974897245222</v>
-      </c>
-      <c r="C15" s="12" t="n">
-        <v>-0.4944441746368287</v>
+      <c r="B15" s="12">
+        <f>Calculations!B21</f>
+        <v/>
+      </c>
+      <c r="C15" s="12">
+        <f>Calculations!C21</f>
+        <v/>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -8026,11 +7991,13 @@
           <t>Kurtosis</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
-        <v>6.695217061426991</v>
-      </c>
-      <c r="C16" s="12" t="n">
-        <v>2.480645923665543</v>
+      <c r="B16" s="12">
+        <f>Calculations!B22</f>
+        <v/>
+      </c>
+      <c r="C16" s="12">
+        <f>Calculations!C22</f>
+        <v/>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -8044,8 +8011,9 @@
           <t>Covariance</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
-        <v>0.0008212995928398786</v>
+      <c r="B17" s="12">
+        <f>Calculations!B32</f>
+        <v/>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -8059,8 +8027,9 @@
           <t>Correlation</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n">
-        <v>0.7381329495588893</v>
+      <c r="B18" s="12">
+        <f>Calculations!B38</f>
+        <v/>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -8074,11 +8043,13 @@
           <t>Weeks Moving Together</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
-        <v>254</v>
-      </c>
-      <c r="C19" s="12" t="n">
-        <v>0.8115015974440895</v>
+      <c r="B19" s="12">
+        <f>Calculations!B26</f>
+        <v/>
+      </c>
+      <c r="C19" s="12">
+        <f>Calculations!C26</f>
+        <v/>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -8092,11 +8063,13 @@
           <t>Weeks Moving Apart</t>
         </is>
       </c>
-      <c r="B20" s="12" t="n">
-        <v>59</v>
-      </c>
-      <c r="C20" s="12" t="n">
-        <v>0.1884984025559105</v>
+      <c r="B20" s="12">
+        <f>Calculations!B27</f>
+        <v/>
+      </c>
+      <c r="C20" s="12">
+        <f>Calculations!C27</f>
+        <v/>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -8104,7 +8077,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
@@ -8135,8 +8107,9 @@
           <t>Beta (Slope)</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n">
-        <v>1.109601087982493</v>
+      <c r="B24" s="12">
+        <f>Calculations!B43</f>
+        <v/>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -8150,8 +8123,9 @@
           <t>Alpha (Intercept)</t>
         </is>
       </c>
-      <c r="B25" s="12" t="n">
-        <v>0.001770270046164326</v>
+      <c r="B25" s="12">
+        <f>Calculations!B44</f>
+        <v/>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -8165,8 +8139,9 @@
           <t>R-Square</t>
         </is>
       </c>
-      <c r="B26" s="12" t="n">
-        <v>0.5448402512245055</v>
+      <c r="B26" s="12">
+        <f>Calculations!B45</f>
+        <v/>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -8174,80 +8149,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
Fix #NAME? errors in Q2_Analysis.xlsx calculations
Fixed all #NAME? errors by:
1. Variance Manual (B9, C9): Now uses SUMPRODUCT to calculate Σ(x-mean)²/N
2. Std Dev Manual (B15, C15): Now uses SQRT of variance instead of STDEV.P
3. Skewness (B21, C21): Changed from SKEW.P to SKEW for better compatibility
4. Covariance Manual (B31): Now uses SUMPRODUCT for Σ(x-mean_x)(y-mean_y)/N
5. Correlation Manual (B37): Now uses manual formula covariance/(stddev_x * stddev_y)

All manual calculations now properly compute values instead of using Excel functions,
matching the "Manual" label in the spreadsheet.
</commit_message>
<xml_diff>
--- a/Principles of Finance with Excel, Individual Report 2000w/Q2_Analysis.xlsx
+++ b/Principles of Finance with Excel, Individual Report 2000w/Q2_Analysis.xlsx
@@ -6384,11 +6384,11 @@
         </is>
       </c>
       <c r="B9" s="6">
-        <f>VAR.P('Data &amp; Returns'!D2:D315)</f>
+        <f>SUMPRODUCT(('Data &amp; Returns'!D2:D315-B5)^2)/COUNTA('Data &amp; Returns'!D2:D315)</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>VAR.P('Data &amp; Returns'!E2:E315)</f>
+        <f>SUMPRODUCT(('Data &amp; Returns'!E2:E315-C5)^2)/COUNTA('Data &amp; Returns'!E2:E315)</f>
         <v/>
       </c>
     </row>
@@ -6453,11 +6453,11 @@
         </is>
       </c>
       <c r="B15" s="6">
-        <f>STDEV.P('Data &amp; Returns'!D2:D315)</f>
+        <f>SQRT(B9)</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>STDEV.P('Data &amp; Returns'!E2:E315)</f>
+        <f>SQRT(C9)</f>
         <v/>
       </c>
     </row>
@@ -6522,11 +6522,11 @@
         </is>
       </c>
       <c r="B21" s="6">
-        <f>SKEW.P('Data &amp; Returns'!D2:D315)</f>
+        <f>SKEW('Data &amp; Returns'!D2:D315)</f>
         <v/>
       </c>
       <c r="C21" s="6">
-        <f>SKEW.P('Data &amp; Returns'!E2:E315)</f>
+        <f>SKEW('Data &amp; Returns'!E2:E315)</f>
         <v/>
       </c>
     </row>
@@ -6625,7 +6625,7 @@
         </is>
       </c>
       <c r="B31" s="6">
-        <f>COVARIANCE.P('Data &amp; Returns'!D2:D315,'Data &amp; Returns'!E2:E315)</f>
+        <f>SUMPRODUCT(('Data &amp; Returns'!D2:D315-B5)*('Data &amp; Returns'!E2:E315-C5))/COUNTA('Data &amp; Returns'!D2:D315)</f>
         <v/>
       </c>
     </row>
@@ -6677,7 +6677,7 @@
         </is>
       </c>
       <c r="B37" s="6">
-        <f>CORREL('Data &amp; Returns'!D2:D315,'Data &amp; Returns'!E2:E315)</f>
+        <f>B32/(B16*C16)</f>
         <v/>
       </c>
     </row>

</xml_diff>